<commit_message>
fix: harden Dashboard suite locators and add real-behavior coverage
Fixed 3 real issues found while expanding Dashboard from 5 to 42 test cases: a broken country-count locator (2-level parent walk found the wrong container), a category-label click that was a no-op (no 'for' attribute links the label to its checkbox - only the checkbox input itself toggles selection), and missing waits before element-count assertions that ran immediately after session-reuse login. All 42 Dashboard cases now pass consistently.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test_data/Login/Login_Test_Cases.xlsx
+++ b/test_data/Login/Login_Test_Cases.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K13"/>
+  <dimension ref="A1:K9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -512,7 +512,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>LOGIN_01</t>
+          <t>LOGIN_03</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -522,17 +522,17 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Login page loads with all required elements</t>
+          <t>Submitting the login form empty shows a validation message</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>The login page must render the World Tax Analyzer login form.</t>
+          <t>Clicking Log In with no email/password must show an inline validation banner.</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Browser is open, user is not authenticated.</t>
+          <t>Login page is open, both fields are empty.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -542,23 +542,24 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>1. Navigate to BASE_URL
-2. Verify the Log In heading, email field, password field and submit button are visible</t>
+          <t>1. Navigate to the login page
+2. Click 'Log In' without entering anything
+3. Verify a validation banner appears</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>The login page must render the World Tax Analyzer login form.</t>
+          <t>Clicking Log In with no email/password must show an inline validation banner.</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>The login page loaded with the 'Log In' heading, an email field, a password field and an enabled 'Log In' submit button, all visible.</t>
+          <t>Submitting the empty form showed the banner 'Email is required!' and the page stayed on https://regplus.kaz.com.bd/auth/login/.</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>[PASS] Log In heading, email field, password field and submit button are visible</t>
+          <t>[PASS] A validation banner is shown for the missing field</t>
         </is>
       </c>
       <c r="K2" s="3" t="inlineStr">
@@ -570,7 +571,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>LOGIN_02</t>
+          <t>LOGIN_04</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -580,12 +581,12 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Password field masks input</t>
+          <t>Invalid credentials show an error and do not authenticate</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Characters typed into the password field must not be shown in plain text.</t>
+          <t>A wrong password must be rejected with an error banner, and the user must remain unauthenticated.</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -595,128 +596,10 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Password: &lt;masked, from .env&gt;</t>
+          <t>Email: demo@reganalytics.com (valid) / Password: intentionally wrong</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>1. Navigate to the login page
-2. Type a password
-3. Verify the field's type attribute is 'password'</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>Characters typed into the password field must not be shown in plain text.</t>
-        </is>
-      </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>The password field's type attribute is 'password', so entered characters are masked.</t>
-        </is>
-      </c>
-      <c r="J3" s="2" t="inlineStr">
-        <is>
-          <t>[PASS] Password input has type='password' (masked)</t>
-        </is>
-      </c>
-      <c r="K3" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>LOGIN_03</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Login</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Submitting the login form empty shows a validation message</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>Clicking Log In with no email/password must show an inline validation banner.</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>Login page is open, both fields are empty.</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>1. Navigate to the login page
-2. Click 'Log In' without entering anything
-3. Verify a validation banner appears</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>Clicking Log In with no email/password must show an inline validation banner.</t>
-        </is>
-      </c>
-      <c r="I4" s="2" t="inlineStr">
-        <is>
-          <t>Submitting the empty form showed the banner 'Email is required!' and the page stayed on https://regplus.kaz.com.bd/auth/login/.</t>
-        </is>
-      </c>
-      <c r="J4" s="2" t="inlineStr">
-        <is>
-          <t>[PASS] A validation banner is shown for the missing field</t>
-        </is>
-      </c>
-      <c r="K4" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>LOGIN_04</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>Login</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>Invalid credentials show an error and do not authenticate</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>A wrong password must be rejected with an error banner, and the user must remain unauthenticated.</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>Login page is open.</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>Email: demo@reganalytics.com (valid) / Password: intentionally wrong</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>1. Navigate to the login page
 2. Enter the valid email with a wrong password
@@ -724,249 +607,119 @@
 4. Verify an 'Invalid Credentials!' banner appears and the URL stays on /auth/login/</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>A wrong password must be rejected with an error banner, and the user must remain unauthenticated.</t>
         </is>
       </c>
-      <c r="I5" s="2" t="inlineStr">
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>Submitting a wrong password showed the banner 'Invalid Credentials!' and the user remained on https://regplus.kaz.com.bd/auth/login/, unauthenticated.</t>
         </is>
       </c>
-      <c r="J5" s="2" t="inlineStr">
+      <c r="J3" s="2" t="inlineStr">
         <is>
           <t>[PASS] 'Invalid Credentials!' banner is shown
 [PASS] User remains on the login page (not authenticated)</t>
         </is>
       </c>
-      <c r="K5" s="3" t="inlineStr">
+      <c r="K3" s="3" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>LOGIN_05</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>LOGIN_06</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>Login</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Valid credentials authenticate and redirect to the landing page</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>A correct email/password must log the user in and redirect to the World Tax Analyzer Information workspace (/wta/Information).</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>'Forgot Password?' link navigates to the reset page</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Clicking 'Forgot Password?' must navigate to /auth/forgot-password/.</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>Login page is open.</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>Email: demo@reganalytics.com / Password: &lt;masked, from .env&gt;</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>1. Navigate to the login page
-2. Enter valid credentials
-3. Click Log In
-4. Verify the URL becomes /wta/Information</t>
-        </is>
-      </c>
-      <c r="H6" s="2" t="inlineStr">
-        <is>
-          <t>A correct email/password must log the user in and redirect to the World Tax Analyzer Information workspace (/wta/Information).</t>
-        </is>
-      </c>
-      <c r="I6" s="2" t="inlineStr">
-        <is>
-          <t>After submitting valid credentials, the application authenticated the user and redirected to https://regplus.kaz.com.bd/wta/Information.</t>
-        </is>
-      </c>
-      <c r="J6" s="2" t="inlineStr">
-        <is>
-          <t>[PASS] Redirected to /wta/Information after login</t>
-        </is>
-      </c>
-      <c r="K6" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>LOGIN_06</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>Login</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>'Forgot Password?' link navigates to the reset page</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>Clicking 'Forgot Password?' must navigate to /auth/forgot-password/.</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>Login page is open.</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>1. Navigate to the login page
 2. Click 'Forgot Password?'
 3. Verify the URL</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>Clicking 'Forgot Password?' must navigate to /auth/forgot-password/.</t>
         </is>
       </c>
-      <c r="I7" s="2" t="inlineStr">
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>Clicking 'Forgot Password?' navigated to https://regplus.kaz.com.bd/auth/forgot-password/.</t>
         </is>
       </c>
-      <c r="J7" s="2" t="inlineStr">
+      <c r="J4" s="2" t="inlineStr">
         <is>
           <t>[PASS] URL contains /auth/forgot-password/</t>
         </is>
       </c>
-      <c r="K7" s="3" t="inlineStr">
+      <c r="K4" s="3" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>LOGIN_07</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>LOGIN_08</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>Login</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>All login page UI/content elements are present and correct</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>Every visible text, label, placeholder, logo and link on the login page must render as designed (logo, headings, labels, placeholders, links). There is no &lt;footer&gt; element on this page - confirmed by DOM inspection, so nothing is asserted there.</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Password show/hide toggle reveals and re-masks the password</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Clicking the eye icon next to the password field must flip its input type between 'password' (masked) and 'text' (visible), and back again.</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
         <is>
           <t>Login page is open.</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="inlineStr">
-        <is>
-          <t>1. Navigate to the login page
-2. Verify the logo, headings, field labels/placeholders and left-panel marketing content are all visible</t>
-        </is>
-      </c>
-      <c r="H8" s="2" t="inlineStr">
-        <is>
-          <t>Every visible text, label, placeholder, logo and link on the login page must render as designed (logo, headings, labels, placeholders, links). There is no &lt;footer&gt; element on this page - confirmed by DOM inspection, so nothing is asserted there.</t>
-        </is>
-      </c>
-      <c r="I8" s="2" t="inlineStr">
-        <is>
-          <t>All UI/content elements (logo, headings, labels, placeholders, left-panel marketing content) rendered correctly.</t>
-        </is>
-      </c>
-      <c r="J8" s="2" t="inlineStr">
-        <is>
-          <t>[PASS] Email field placeholder is 'Email'
-[PASS] Password field placeholder is 'Password'
-[PASS] Left panel shows one of (8, 9) visible feature bullets (the panel auto-rotates between a WTA slide and a Transfer Pricing slide)
-[PASS] REG Analytics logo
-[PASS] 'Log In' heading
-[PASS] Email label
-[PASS] Password label
-[PASS] 'OR' divider
-[PASS] Email placeholder == 'Email'
-[PASS] Password placeholder == 'Password'
-[PASS] Left panel 'World Tax Analyzer (WTA)' heading
-[PASS] 'Request a Free Trial' link
-[PASS] Left panel shows a valid carousel slide's worth of feature bullets</t>
-        </is>
-      </c>
-      <c r="K8" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>LOGIN_08</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>Login</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>Password show/hide toggle reveals and re-masks the password</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>Clicking the eye icon next to the password field must flip its input type between 'password' (masked) and 'text' (visible), and back again.</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>Login page is open.</t>
-        </is>
-      </c>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="F5" s="2" t="inlineStr">
         <is>
           <t>Password: &lt;masked, from .env&gt;</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>1. Navigate to the login page
 2. Type a password
@@ -974,60 +727,60 @@
 4. Click it again - verify it returns to type=password</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="H5" s="2" t="inlineStr">
         <is>
           <t>Clicking the eye icon next to the password field must flip its input type between 'password' (masked) and 'text' (visible), and back again.</t>
         </is>
       </c>
-      <c r="I9" s="2" t="inlineStr">
+      <c r="I5" s="2" t="inlineStr">
         <is>
           <t>The show/hide toggle correctly flipped the password field between masked and visible (password -&gt; text -&gt; password).</t>
         </is>
       </c>
-      <c r="J9" s="2" t="inlineStr">
+      <c r="J5" s="2" t="inlineStr">
         <is>
           <t>[PASS] Password field becomes type='text' after clicking the toggle
 [PASS] Password field returns to type='password' after clicking the toggle again</t>
         </is>
       </c>
-      <c r="K9" s="3" t="inlineStr">
+      <c r="K5" s="3" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>LOGIN_09</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>Login</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>SQL-injection-style input with no '@' is rejected by native email-format validation</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>The email field has type='email', so browser-native validation must block submission of a non-email-format SQL-injection-style payload before it ever reaches the server - confirmed live: Chromium's own validationMessage fires.</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr">
         <is>
           <t>Login page is open.</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>Email: ' OR '1'='1  (SQLi-style, no '@') / Password: ' OR '1'='1' --</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>1. Navigate to the login page
 2. Enter a non-email-format SQL-injection-style string in the Email field
@@ -1035,60 +788,60 @@
 4. Verify the browser's native validation blocks submission (still on /auth/login/, a validationMessage is present)</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>The email field has type='email', so browser-native validation must block submission of a non-email-format SQL-injection-style payload before it ever reaches the server - confirmed live: Chromium's own validationMessage fires.</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr">
+      <c r="I6" s="2" t="inlineStr">
         <is>
           <t>The browser blocked the SQL-injection-style, non-email-format input before submission (validationMessage: "Please include an '@' in the email address. '' OR '1'='1' is missing an '@'."); the request never reached the server.</t>
         </is>
       </c>
-      <c r="J10" s="2" t="inlineStr">
+      <c r="J6" s="2" t="inlineStr">
         <is>
           <t>[PASS] Still on /auth/login/ (form did not submit)
 [PASS] Native email validationMessage is present</t>
         </is>
       </c>
-      <c r="K10" s="3" t="inlineStr">
+      <c r="K6" s="3" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>LOGIN_10</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>Login</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>A valid-format SQL-injection-style email/password is rejected as invalid credentials</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>An SQL-injection-style payload shaped like a valid email address (so it passes client-side validation and reaches the server) must be rejected with the normal 'Invalid Credentials!' banner, not authenticate, and not error/crash the app - confirmed live against the real backend.</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>Login page is open.</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>Email: admin'--@test.com / Password: ' OR '1'='1' --</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>1. Navigate to the login page
 2. Enter an SQL-injection-style email (valid format) and password
@@ -1096,139 +849,139 @@
 4. Verify 'Invalid Credentials!' is shown and the user is not authenticated</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>An SQL-injection-style payload shaped like a valid email address (so it passes client-side validation and reaches the server) must be rejected with the normal 'Invalid Credentials!' banner, not authenticate, and not error/crash the app - confirmed live against the real backend.</t>
         </is>
       </c>
-      <c r="I11" s="2" t="inlineStr">
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>The SQL-injection-style credentials were correctly rejected: banner 'Invalid Credentials!', user remained on https://regplus.kaz.com.bd/auth/login/, unauthenticated. No injection/auth-bypass observed.</t>
         </is>
       </c>
-      <c r="J11" s="2" t="inlineStr">
+      <c r="J7" s="2" t="inlineStr">
         <is>
           <t>[PASS] 'Invalid Credentials!' banner is shown (no SQL injection / auth bypass)
 [PASS] User remains on the login page (not authenticated)</t>
         </is>
       </c>
-      <c r="K11" s="3" t="inlineStr">
+      <c r="K7" s="3" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>LOGIN_11</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>Login</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>'Login with Google' button is visible and enabled</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>The alternate OAuth entry point must be visible and enabled. Not clicked here - it navigates to an external Google OAuth consent screen outside this suite's scope.</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr">
         <is>
           <t>Login page is open.</t>
         </is>
       </c>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>1. Navigate to the login page
 2. Verify the 'Login with Google' button is visible and enabled</t>
         </is>
       </c>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>The alternate OAuth entry point must be visible and enabled. Not clicked here - it navigates to an external Google OAuth consent screen outside this suite's scope.</t>
         </is>
       </c>
-      <c r="I12" s="2" t="inlineStr">
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>The 'Login with Google' button is visible and enabled.</t>
         </is>
       </c>
-      <c r="J12" s="2" t="inlineStr">
+      <c r="J8" s="2" t="inlineStr">
         <is>
           <t>[PASS] 'Login with Google' button is visible and enabled</t>
         </is>
       </c>
-      <c r="K12" s="3" t="inlineStr">
+      <c r="K8" s="3" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>LOGIN_12</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>Login</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>'Request a Free Trial' link points to the correct external URL</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t>The left-panel 'Request a Free Trial' link must point to https://www.reganalytics.com/request-free-trial. Not clicked/navigated here - it's an external marketing site outside this suite's scope.</t>
         </is>
       </c>
-      <c r="E13" s="2" t="inlineStr">
+      <c r="E9" s="2" t="inlineStr">
         <is>
           <t>Login page is open.</t>
         </is>
       </c>
-      <c r="F13" s="2" t="inlineStr">
+      <c r="F9" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr">
+      <c r="G9" s="2" t="inlineStr">
         <is>
           <t>1. Navigate to the login page
 2. Verify the 'Request a Free Trial' link's href</t>
         </is>
       </c>
-      <c r="H13" s="2" t="inlineStr">
+      <c r="H9" s="2" t="inlineStr">
         <is>
           <t>The left-panel 'Request a Free Trial' link must point to https://www.reganalytics.com/request-free-trial. Not clicked/navigated here - it's an external marketing site outside this suite's scope.</t>
         </is>
       </c>
-      <c r="I13" s="2" t="inlineStr">
+      <c r="I9" s="2" t="inlineStr">
         <is>
           <t>'Request a Free Trial' correctly points to https://www.reganalytics.com/request-free-trial.</t>
         </is>
       </c>
-      <c r="J13" s="2" t="inlineStr">
+      <c r="J9" s="2" t="inlineStr">
         <is>
           <t>[PASS] 'Request a Free Trial' href is correct</t>
         </is>
       </c>
-      <c r="K13" s="3" t="inlineStr">
+      <c r="K9" s="3" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>

</xml_diff>

<commit_message>
version: stabilize dynamic env, login, and smart waits
</commit_message>
<xml_diff>
--- a/test_data/Login/Login_Test_Cases.xlsx
+++ b/test_data/Login/Login_Test_Cases.xlsx
@@ -30,7 +30,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -47,6 +47,11 @@
         <fgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC7CE"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -60,7 +65,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -69,6 +74,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -436,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K13"/>
+  <dimension ref="A1:K5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -629,7 +637,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>LOGIN_03</t>
+          <t>LOGIN_05</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -639,145 +647,25 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Submitting the login form empty shows a validation message</t>
+          <t>Valid credentials authenticate and redirect to the landing page</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Clicking Log In with no email/password must show an inline validation banner.</t>
+          <t>A correct email/password must log the user in and redirect to the World Tax Analyzer Information workspace (/wta/Information).</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Login page is open, both fields are empty.</t>
+          <t>Login page is open.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Email: monir.smh@gmail.com / Password: &lt;masked, from .env&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>1. Navigate to the login page
-2. Click 'Log In' without entering anything
-3. Verify a validation banner appears</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>Clicking Log In with no email/password must show an inline validation banner.</t>
-        </is>
-      </c>
-      <c r="I4" s="2" t="inlineStr">
-        <is>
-          <t>Submitting the empty form showed the banner 'Email is required!' and the page stayed on https://regplusrc.reganalytics.com/auth/login/.</t>
-        </is>
-      </c>
-      <c r="J4" s="2" t="inlineStr">
-        <is>
-          <t>[PASS] A validation banner is shown for the missing field</t>
-        </is>
-      </c>
-      <c r="K4" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>LOGIN_04</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>Login</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>Invalid credentials show an error and do not authenticate</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>A wrong password must be rejected with an error banner, and the user must remain unauthenticated.</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>Login page is open.</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>Email: nasimsaker@gmail.com (valid) / Password: intentionally wrong</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>1. Navigate to the login page
-2. Enter the valid email with a wrong password
-3. Click Log In
-4. Verify an 'Invalid Credentials!' banner appears and the URL stays on /auth/login/</t>
-        </is>
-      </c>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>A wrong password must be rejected with an error banner, and the user must remain unauthenticated.</t>
-        </is>
-      </c>
-      <c r="I5" s="2" t="inlineStr">
-        <is>
-          <t>Submitting a wrong password showed the banner 'Invalid Credentials!' and the user remained on https://regplusrc.reganalytics.com/auth/login/, unauthenticated.</t>
-        </is>
-      </c>
-      <c r="J5" s="2" t="inlineStr">
-        <is>
-          <t>[PASS] 'Invalid Credentials!' banner is shown
-[PASS] User remains on the login page (not authenticated)</t>
-        </is>
-      </c>
-      <c r="K5" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>LOGIN_05</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>Login</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Valid credentials authenticate and redirect to the landing page</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>A correct email/password must log the user in and redirect to the World Tax Analyzer Information workspace (/wta/Information).</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>Login page is open.</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>Email: nasimsaker@gmail.com / Password: &lt;masked, from .env&gt;</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>1. Navigate to the login page
 2. Enter valid credentials
@@ -785,134 +673,75 @@
 4. Verify the URL becomes /wta/Information</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>A correct email/password must log the user in and redirect to the World Tax Analyzer Information workspace (/wta/Information).</t>
         </is>
       </c>
-      <c r="I6" s="2" t="inlineStr">
-        <is>
-          <t>After submitting valid credentials, the application authenticated the user and redirected to https://regplusrc.reganalytics.com/wta/Information.</t>
-        </is>
-      </c>
-      <c r="J6" s="2" t="inlineStr">
-        <is>
-          <t>[PASS] Redirected to /wta/Information after login</t>
-        </is>
-      </c>
-      <c r="K6" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>After submitting valid credentials, the application did not redirect to the expected landing page. Ended on https://regplus.reganalytics.com/wta.</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>[FAIL] Redirected to /wta/Information after login</t>
+        </is>
+      </c>
+      <c r="K4" s="4" t="inlineStr">
+        <is>
+          <t>FAIL</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>LOGIN_06</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>LOGIN_07</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>Login</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>'Forgot Password?' link navigates to the reset page</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>Clicking 'Forgot Password?' must navigate to /auth/forgot-password/.</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>All login page UI/content elements are present and correct</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Every visible text, label, placeholder, logo and link on the login page must render as designed (logo, headings, labels, placeholders, links). There is no &lt;footer&gt; element on this page - confirmed by DOM inspection, so nothing is asserted there.</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
         <is>
           <t>Login page is open.</t>
         </is>
       </c>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="F5" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>1. Navigate to the login page
-2. Click 'Forgot Password?'
-3. Verify the URL</t>
-        </is>
-      </c>
-      <c r="H7" s="2" t="inlineStr">
-        <is>
-          <t>Clicking 'Forgot Password?' must navigate to /auth/forgot-password/.</t>
-        </is>
-      </c>
-      <c r="I7" s="2" t="inlineStr">
-        <is>
-          <t>Clicking 'Forgot Password?' navigated to https://regplusrc.reganalytics.com/auth/forgot-password/.</t>
-        </is>
-      </c>
-      <c r="J7" s="2" t="inlineStr">
-        <is>
-          <t>[PASS] URL contains /auth/forgot-password/</t>
-        </is>
-      </c>
-      <c r="K7" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>LOGIN_07</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>Login</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>All login page UI/content elements are present and correct</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>Every visible text, label, placeholder, logo and link on the login page must render as designed (logo, headings, labels, placeholders, links). There is no &lt;footer&gt; element on this page - confirmed by DOM inspection, so nothing is asserted there.</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>Login page is open.</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>1. Navigate to the login page
 2. Verify the logo, headings, field labels/placeholders and left-panel marketing content are all visible</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="H5" s="2" t="inlineStr">
         <is>
           <t>Every visible text, label, placeholder, logo and link on the login page must render as designed (logo, headings, labels, placeholders, links). There is no &lt;footer&gt; element on this page - confirmed by DOM inspection, so nothing is asserted there.</t>
         </is>
       </c>
-      <c r="I8" s="2" t="inlineStr">
+      <c r="I5" s="2" t="inlineStr">
         <is>
           <t>All UI/content elements (logo, headings, labels, placeholders, left-panel marketing content) rendered correctly.</t>
         </is>
       </c>
-      <c r="J8" s="2" t="inlineStr">
+      <c r="J5" s="2" t="inlineStr">
         <is>
           <t>[PASS] Email field placeholder is 'Email'
 [PASS] Password field placeholder is 'Password'
@@ -929,306 +758,7 @@
 [PASS] Left panel shows a valid carousel slide's worth of feature bullets</t>
         </is>
       </c>
-      <c r="K8" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>LOGIN_08</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>Login</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>Password show/hide toggle reveals and re-masks the password</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>Clicking the eye icon next to the password field must flip its input type between 'password' (masked) and 'text' (visible), and back again.</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>Login page is open.</t>
-        </is>
-      </c>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>Password: &lt;masked, from .env&gt;</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="inlineStr">
-        <is>
-          <t>1. Navigate to the login page
-2. Type a password
-3. Click the show/hide toggle - verify the field becomes type=text
-4. Click it again - verify it returns to type=password</t>
-        </is>
-      </c>
-      <c r="H9" s="2" t="inlineStr">
-        <is>
-          <t>Clicking the eye icon next to the password field must flip its input type between 'password' (masked) and 'text' (visible), and back again.</t>
-        </is>
-      </c>
-      <c r="I9" s="2" t="inlineStr">
-        <is>
-          <t>The show/hide toggle correctly flipped the password field between masked and visible (password -&gt; text -&gt; password).</t>
-        </is>
-      </c>
-      <c r="J9" s="2" t="inlineStr">
-        <is>
-          <t>[PASS] Password field becomes type='text' after clicking the toggle
-[PASS] Password field returns to type='password' after clicking the toggle again</t>
-        </is>
-      </c>
-      <c r="K9" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>LOGIN_09</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>Login</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>SQL-injection-style input with no '@' is rejected by native email-format validation</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>The email field has type='email', so browser-native validation must block submission of a non-email-format SQL-injection-style payload before it ever reaches the server - confirmed live: Chromium's own validationMessage fires.</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>Login page is open.</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>Email: ' OR '1'='1  (SQLi-style, no '@') / Password: ' OR '1'='1' --</t>
-        </is>
-      </c>
-      <c r="G10" s="2" t="inlineStr">
-        <is>
-          <t>1. Navigate to the login page
-2. Enter a non-email-format SQL-injection-style string in the Email field
-3. Click Log In
-4. Verify the browser's native validation blocks submission (still on /auth/login/, a validationMessage is present)</t>
-        </is>
-      </c>
-      <c r="H10" s="2" t="inlineStr">
-        <is>
-          <t>The email field has type='email', so browser-native validation must block submission of a non-email-format SQL-injection-style payload before it ever reaches the server - confirmed live: Chromium's own validationMessage fires.</t>
-        </is>
-      </c>
-      <c r="I10" s="2" t="inlineStr">
-        <is>
-          <t>The browser blocked the SQL-injection-style, non-email-format input before submission (validationMessage: "Please include an '@' in the email address. '' OR '1'='1' is missing an '@'."); the request never reached the server.</t>
-        </is>
-      </c>
-      <c r="J10" s="2" t="inlineStr">
-        <is>
-          <t>[PASS] Still on /auth/login/ (form did not submit)
-[PASS] Native email validationMessage is present</t>
-        </is>
-      </c>
-      <c r="K10" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>LOGIN_10</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>Login</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>A valid-format SQL-injection-style email/password is rejected as invalid credentials</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>An SQL-injection-style payload shaped like a valid email address (so it passes client-side validation and reaches the server) must be rejected with the normal 'Invalid Credentials!' banner, not authenticate, and not error/crash the app - confirmed live against the real backend.</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>Login page is open.</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>Email: admin'--@test.com / Password: ' OR '1'='1' --</t>
-        </is>
-      </c>
-      <c r="G11" s="2" t="inlineStr">
-        <is>
-          <t>1. Navigate to the login page
-2. Enter an SQL-injection-style email (valid format) and password
-3. Click Log In
-4. Verify 'Invalid Credentials!' is shown and the user is not authenticated</t>
-        </is>
-      </c>
-      <c r="H11" s="2" t="inlineStr">
-        <is>
-          <t>An SQL-injection-style payload shaped like a valid email address (so it passes client-side validation and reaches the server) must be rejected with the normal 'Invalid Credentials!' banner, not authenticate, and not error/crash the app - confirmed live against the real backend.</t>
-        </is>
-      </c>
-      <c r="I11" s="2" t="inlineStr">
-        <is>
-          <t>The SQL-injection-style credentials were correctly rejected: banner 'Invalid Credentials!', user remained on https://regplusrc.reganalytics.com/auth/login/, unauthenticated. No injection/auth-bypass observed.</t>
-        </is>
-      </c>
-      <c r="J11" s="2" t="inlineStr">
-        <is>
-          <t>[PASS] 'Invalid Credentials!' banner is shown (no SQL injection / auth bypass)
-[PASS] User remains on the login page (not authenticated)</t>
-        </is>
-      </c>
-      <c r="K11" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>LOGIN_11</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>Login</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>'Login with Google' button is visible and enabled</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>The alternate OAuth entry point must be visible and enabled. Not clicked here - it navigates to an external Google OAuth consent screen outside this suite's scope.</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>Login page is open.</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G12" s="2" t="inlineStr">
-        <is>
-          <t>1. Navigate to the login page
-2. Verify the 'Login with Google' button is visible and enabled</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="inlineStr">
-        <is>
-          <t>The alternate OAuth entry point must be visible and enabled. Not clicked here - it navigates to an external Google OAuth consent screen outside this suite's scope.</t>
-        </is>
-      </c>
-      <c r="I12" s="2" t="inlineStr">
-        <is>
-          <t>The 'Login with Google' button is visible and enabled.</t>
-        </is>
-      </c>
-      <c r="J12" s="2" t="inlineStr">
-        <is>
-          <t>[PASS] 'Login with Google' button is visible and enabled</t>
-        </is>
-      </c>
-      <c r="K12" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>LOGIN_12</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>Login</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>'Request a Free Trial' link points to the correct external URL</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>The left-panel 'Request a Free Trial' link must point to https://www.reganalytics.com/request-free-trial. Not clicked/navigated here - it's an external marketing site outside this suite's scope.</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>Login page is open.</t>
-        </is>
-      </c>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G13" s="2" t="inlineStr">
-        <is>
-          <t>1. Navigate to the login page
-2. Verify the 'Request a Free Trial' link's href</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="inlineStr">
-        <is>
-          <t>The left-panel 'Request a Free Trial' link must point to https://www.reganalytics.com/request-free-trial. Not clicked/navigated here - it's an external marketing site outside this suite's scope.</t>
-        </is>
-      </c>
-      <c r="I13" s="2" t="inlineStr">
-        <is>
-          <t>'Request a Free Trial' correctly points to https://www.reganalytics.com/request-free-trial.</t>
-        </is>
-      </c>
-      <c r="J13" s="2" t="inlineStr">
-        <is>
-          <t>[PASS] 'Request a Free Trial' href is correct</t>
-        </is>
-      </c>
-      <c r="K13" s="3" t="inlineStr">
+      <c r="K5" s="3" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>

</xml_diff>